<commit_message>
add | new data column traffic_flow in tb_machine
</commit_message>
<xml_diff>
--- a/frontend/public/Mau_Excel_MayMoc.xlsx
+++ b/frontend/public/Mau_Excel_MayMoc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\react\TPM\frontend\public\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\react\tpm\frontend\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88E98A48-0F65-4DB4-9E60-B8D520DE3C79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2435EA43-0994-40D3-8E78-2118619C6F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DanhSachMayMoc" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t>Serial</t>
   </si>
@@ -126,16 +126,19 @@
     <t>20x30</t>
   </si>
   <si>
-    <t>Công suất</t>
-  </si>
-  <si>
-    <t>Áp suất</t>
-  </si>
-  <si>
-    <t>Điện áp</t>
-  </si>
-  <si>
     <t>GIANG THÀNH</t>
+  </si>
+  <si>
+    <t>Công suất (W)</t>
+  </si>
+  <si>
+    <t>Áp suất (MPa)</t>
+  </si>
+  <si>
+    <t>Điện áp (V)</t>
+  </si>
+  <si>
+    <t>Lưu lượng khí nén (lít/phút)</t>
   </si>
 </sst>
 </file>
@@ -559,29 +562,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" customWidth="1"/>
-    <col min="4" max="4" width="30.28515625" customWidth="1"/>
+    <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="22.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" hidden="1"/>
+    <col min="9" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -607,31 +610,34 @@
         <v>20</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -648,7 +654,7 @@
         <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
         <v>12</v>
@@ -665,23 +671,26 @@
       <c r="K2">
         <v>20</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2">
+        <v>20</v>
+      </c>
+      <c r="M2" s="3">
         <v>150000000</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>13</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>10</v>
       </c>
-      <c r="O2" s="3">
+      <c r="P2" s="3">
         <v>150000000</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -698,7 +707,7 @@
         <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G3" t="s">
         <v>17</v>
@@ -706,26 +715,26 @@
       <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="3">
+      <c r="M3" s="3">
         <v>5000000</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>18</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>5</v>
       </c>
-      <c r="O3" s="3">
+      <c r="P3" s="3">
         <v>5000000</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="L1:P1 L2:N3 P2:P3 A2:A3 D2:D3 G1:G3 D1:E1 A1:B1" numberStoredAsText="1"/>
+    <ignoredError sqref="M1:Q1 M2:O3 Q2:Q3 A2:A3 D2:D3 G1:G3 D1:E1 A1:B1" numberStoredAsText="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>